<commit_message>
#261022 fix: fixed global settings
</commit_message>
<xml_diff>
--- a/files/black-list.xlsx
+++ b/files/black-list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koray.zorlu\projects\arierp\arierp_backend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD18CD3-A44A-4F4E-833F-8FDAA04A7F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB27AB41-E0D4-4B1D-8C5F-F9883D9393A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{3BBC1162-E7B6-4495-BD4F-07E3B07D0A73}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BBC1162-E7B6-4495-BD4F-07E3B07D0A73}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="121">
   <si>
     <t>TC/VKN/Pasaport No</t>
   </si>
@@ -59,694 +59,346 @@
     <t>Resmi Gazete Tarih ve Sayısı</t>
   </si>
   <si>
-    <t>ERDEM ÖZKAN</t>
-  </si>
-  <si>
-    <t>15914988634</t>
-  </si>
-  <si>
-    <t>GÖKAY YILMAZ</t>
-  </si>
-  <si>
-    <t>28756103608</t>
-  </si>
-  <si>
-    <t>İZZET GÖKHAN ÖZBİLGİN</t>
-  </si>
-  <si>
-    <t>18559796886</t>
-  </si>
-  <si>
-    <t>SERDAR ORMAN</t>
-  </si>
-  <si>
-    <t>24218375248</t>
-  </si>
-  <si>
-    <t>YASEMİN ÖZYURT</t>
-  </si>
-  <si>
-    <t>23438015422</t>
-  </si>
-  <si>
-    <t>ABDURRAHMAN KOCA</t>
-  </si>
-  <si>
-    <t>18848573532</t>
-  </si>
-  <si>
-    <t>BURÇKAN KAPLAN</t>
-  </si>
-  <si>
-    <t>15062869298</t>
-  </si>
-  <si>
-    <t>CAN DEMİRKOL</t>
-  </si>
-  <si>
-    <t>15760992908</t>
-  </si>
-  <si>
-    <t>ÇAĞLA KELLE</t>
-  </si>
-  <si>
-    <t>18619912546</t>
-  </si>
-  <si>
-    <t>DENİZ İNAN</t>
-  </si>
-  <si>
-    <t>26518188122</t>
-  </si>
-  <si>
-    <t>HANİFE AYDIN</t>
-  </si>
-  <si>
-    <t>14540297530</t>
-  </si>
-  <si>
-    <t>İLKER BAYRAKTAR</t>
-  </si>
-  <si>
-    <t>35921089254</t>
-  </si>
-  <si>
-    <t>İSMAİL CANIPEK</t>
-  </si>
-  <si>
-    <t>23660229864</t>
-  </si>
-  <si>
-    <t>KADİR BERKAY AYTEKİN</t>
-  </si>
-  <si>
-    <t>29491458282</t>
-  </si>
-  <si>
-    <t>KADİR SAKALLIOĞLU</t>
-  </si>
-  <si>
-    <t>17419181046</t>
-  </si>
-  <si>
-    <t>KEMAL AKKAYA</t>
-  </si>
-  <si>
-    <t>19969023302</t>
-  </si>
-  <si>
-    <t>KUBİLAY ÖZYURT</t>
-  </si>
-  <si>
-    <t>64657220068</t>
-  </si>
-  <si>
-    <t>MAHİR CAN EREREN</t>
-  </si>
-  <si>
-    <t>12515459754</t>
-  </si>
-  <si>
-    <t>METE MUZAFFER BIÇAKLIOĞLU</t>
-  </si>
-  <si>
-    <t>34768622020</t>
-  </si>
-  <si>
-    <t>MUSTAFA AKYOL</t>
-  </si>
-  <si>
-    <t>35071847780</t>
-  </si>
-  <si>
-    <t>ÖZGÜ MIZIRAKCI</t>
-  </si>
-  <si>
-    <t>18320050346</t>
-  </si>
-  <si>
-    <t>REYHAN YILMAZ</t>
-  </si>
-  <si>
-    <t>45586817598</t>
-  </si>
-  <si>
-    <t>SADIK MURAT BARIŞIK</t>
-  </si>
-  <si>
-    <t>31210845228</t>
-  </si>
-  <si>
-    <t>SÜLEYMAN AYGÜN</t>
-  </si>
-  <si>
-    <t>24674534678</t>
-  </si>
-  <si>
-    <t>TARIK İŞAT</t>
-  </si>
-  <si>
-    <t>22481165368</t>
-  </si>
-  <si>
-    <t>TUĞBA BALÇIK AYTAN</t>
-  </si>
-  <si>
-    <t>10291241976</t>
-  </si>
-  <si>
-    <t>UĞUR AKBULUT</t>
-  </si>
-  <si>
-    <t>19955244650</t>
-  </si>
-  <si>
-    <t>MEHMET FATİH GÖKALP</t>
-  </si>
-  <si>
-    <t>32500804406</t>
-  </si>
-  <si>
-    <t>MEHMET NURİ GÖKALP</t>
-  </si>
-  <si>
-    <t>32503804342</t>
-  </si>
-  <si>
-    <t>MEHMET ZİYA GÖKALP</t>
-  </si>
-  <si>
-    <t>32551802758</t>
-  </si>
-  <si>
-    <t>NAMIK KEMAL GÖKALP</t>
-  </si>
-  <si>
-    <t>32545802986</t>
-  </si>
-  <si>
-    <t>SİBEL GÖKALP</t>
-  </si>
-  <si>
-    <t>29296644316</t>
-  </si>
-  <si>
-    <t>SÜLEYMAN ARPASLAN</t>
-  </si>
-  <si>
-    <t>25330080898</t>
-  </si>
-  <si>
-    <t>EBRU AVCI</t>
-  </si>
-  <si>
-    <t>30862121834</t>
-  </si>
-  <si>
-    <t>ENDER ÖLMEZ</t>
-  </si>
-  <si>
-    <t>46237676618</t>
-  </si>
-  <si>
-    <t>HAKAN ERDOĞAN</t>
-  </si>
-  <si>
-    <t>33562107580</t>
-  </si>
-  <si>
-    <t>KAAN YILMAZ</t>
-  </si>
-  <si>
-    <t>46588925120</t>
-  </si>
-  <si>
-    <t>KADER SARIGÜL</t>
-  </si>
-  <si>
-    <t>58804449204</t>
-  </si>
-  <si>
-    <t>NEBİHE DOĞANLAR</t>
-  </si>
-  <si>
-    <t>28211478036</t>
-  </si>
-  <si>
-    <t>ÖMER ERYILMAZ</t>
-  </si>
-  <si>
-    <t>15656133392</t>
-  </si>
-  <si>
-    <t>ŞEMSİHAN KARACA</t>
-  </si>
-  <si>
-    <t>49471628078</t>
-  </si>
-  <si>
-    <t>TUBA KONUKSEVER UYSAL</t>
-  </si>
-  <si>
-    <t>45772958074</t>
-  </si>
-  <si>
-    <t>YASİN ÇETİN</t>
-  </si>
-  <si>
-    <t>22010555820</t>
-  </si>
-  <si>
-    <t>SAİT AYTAÇ</t>
-  </si>
-  <si>
-    <t>39847193880</t>
-  </si>
-  <si>
-    <t>SERDAR TURHAN</t>
-  </si>
-  <si>
-    <t>16549659500</t>
-  </si>
-  <si>
-    <t>AHMET SELİM BAYCIN</t>
-  </si>
-  <si>
-    <t>10870679862</t>
-  </si>
-  <si>
-    <t>ALİ BAKAÇ</t>
-  </si>
-  <si>
-    <t>27886019742</t>
-  </si>
-  <si>
-    <t>BARIŞ ENİŞ</t>
-  </si>
-  <si>
-    <t>37642292746</t>
-  </si>
-  <si>
-    <t>FURKAN ÇETİNKAYA</t>
-  </si>
-  <si>
-    <t>46600321978</t>
-  </si>
-  <si>
-    <t>İSMAİL BİCİK</t>
-  </si>
-  <si>
-    <t>43007098540</t>
-  </si>
-  <si>
-    <t>MECİT BATUHAN ALPMAN</t>
-  </si>
-  <si>
-    <t>20174204998</t>
-  </si>
-  <si>
-    <t>SELMA YÜKSEL</t>
-  </si>
-  <si>
-    <t>50113307022</t>
-  </si>
-  <si>
-    <t>SEVNUR CAN</t>
-  </si>
-  <si>
-    <t>22771392092</t>
-  </si>
-  <si>
-    <t>TARKAN KIROĞLU</t>
-  </si>
-  <si>
-    <t>23810551128</t>
-  </si>
-  <si>
-    <t>YAVUZ YAPRAK</t>
-  </si>
-  <si>
-    <t>29650347792</t>
-  </si>
-  <si>
-    <t>AYŞEGÜL KAYA</t>
-  </si>
-  <si>
-    <t>30889508922</t>
-  </si>
-  <si>
-    <t>BÜLENT UYGUN</t>
-  </si>
-  <si>
-    <t>34531590358</t>
-  </si>
-  <si>
-    <t>ERDİN ÖZEL</t>
-  </si>
-  <si>
-    <t>46303142160</t>
-  </si>
-  <si>
-    <t>ETHEM UMUT BEYTORUN</t>
-  </si>
-  <si>
-    <t>27158032424</t>
-  </si>
-  <si>
-    <t>EVREN UÇAR</t>
-  </si>
-  <si>
-    <t>38671108374</t>
-  </si>
-  <si>
-    <t>HAKAN AHMET UZUN</t>
-  </si>
-  <si>
-    <t>35287788402</t>
-  </si>
-  <si>
-    <t>İBRAHİM BEKCİ</t>
-  </si>
-  <si>
-    <t>11414290338</t>
-  </si>
-  <si>
-    <t>SERKAN KARAKAŞ</t>
-  </si>
-  <si>
-    <t>23330136898</t>
-  </si>
-  <si>
-    <t>CEM GÜRKAN ALPAY</t>
-  </si>
-  <si>
-    <t>55006428044</t>
-  </si>
-  <si>
-    <t>ELİF ÖZÜŞ</t>
-  </si>
-  <si>
-    <t>19270355888</t>
-  </si>
-  <si>
-    <t>EMİR MÜNİR SARPYENER</t>
-  </si>
-  <si>
-    <t>30406884126</t>
-  </si>
-  <si>
-    <t>EMRE TEZMEN</t>
-  </si>
-  <si>
-    <t>10349542222</t>
-  </si>
-  <si>
-    <t>EMRULLAH FURKAN GÜN</t>
-  </si>
-  <si>
-    <t>45274614508</t>
-  </si>
-  <si>
     <t>GÜL AYŞE ÇOLAK</t>
   </si>
   <si>
-    <t>28189250566</t>
-  </si>
-  <si>
     <t>MUHAMMED TALHA SAZAK</t>
   </si>
   <si>
-    <t>13639129622</t>
-  </si>
-  <si>
     <t>OĞUZ TEZMEN</t>
   </si>
   <si>
-    <t>10364541712</t>
-  </si>
-  <si>
     <t>TOLGA DIRAMALIOL</t>
   </si>
   <si>
-    <t>41875472424</t>
-  </si>
-  <si>
     <t>ENVER ÇEVİK</t>
   </si>
   <si>
-    <t>25984674948</t>
-  </si>
-  <si>
     <t>MAHMUT KORKMAZ</t>
   </si>
   <si>
-    <t>34031356454</t>
-  </si>
-  <si>
     <t>MUHAMMED YARIZ</t>
   </si>
   <si>
-    <t>22618757558</t>
-  </si>
-  <si>
     <t>ABDULLAH ERCAN</t>
   </si>
   <si>
-    <t>10285120492</t>
-  </si>
-  <si>
     <t>MELİS SANDAL</t>
   </si>
   <si>
-    <t>36616642778</t>
-  </si>
-  <si>
     <t>EMRULLAH ERCAN</t>
   </si>
   <si>
-    <t>10312119536</t>
-  </si>
-  <si>
     <t>ÖMER BEDİR ÇETİNEL</t>
   </si>
   <si>
-    <t>14291640388</t>
-  </si>
-  <si>
     <t>MUSTAFA DEDİK</t>
   </si>
   <si>
-    <t>26881948590</t>
-  </si>
-  <si>
     <t>HAKAN YILDIZ</t>
   </si>
   <si>
-    <t>44173337372</t>
-  </si>
-  <si>
     <t>ENVER GEÇGEL</t>
   </si>
   <si>
-    <t>44086958824</t>
-  </si>
-  <si>
     <t>İSMET ÖĞÜT</t>
   </si>
   <si>
-    <t>64813347264</t>
-  </si>
-  <si>
     <t>TARZAN TARIK SARVAN</t>
   </si>
   <si>
-    <t>51073602172</t>
-  </si>
-  <si>
     <t>TOLGA AYDİN</t>
   </si>
   <si>
-    <t>47323812538</t>
-  </si>
-  <si>
     <t>EZGİ KAYA</t>
   </si>
   <si>
-    <t>13390316040</t>
-  </si>
-  <si>
     <t>BURHAN TUNÇ ÖZKAN</t>
   </si>
   <si>
-    <t>14914235908</t>
-  </si>
-  <si>
     <t>MEHMET SELÇUK AKSOY</t>
   </si>
   <si>
-    <t>25870676674</t>
-  </si>
-  <si>
     <t>TURGAY CEYLANİ</t>
   </si>
   <si>
-    <t>18146324638</t>
-  </si>
-  <si>
     <t>RIZA KANDEMİR</t>
   </si>
   <si>
-    <t>10262056530</t>
-  </si>
-  <si>
     <t>CENGİZ AVCI</t>
   </si>
   <si>
-    <t>51949688088</t>
-  </si>
-  <si>
     <t>FURKAN TALAY</t>
   </si>
   <si>
-    <t>63514100796</t>
-  </si>
-  <si>
     <t>METEHAN ÜLGENER</t>
   </si>
   <si>
-    <t>11299087108</t>
-  </si>
-  <si>
     <t>ALİ YILDIZ</t>
   </si>
   <si>
-    <t>45235539758</t>
-  </si>
-  <si>
     <t>KAZİM KOCAPINAR</t>
   </si>
   <si>
-    <t>39611154796</t>
-  </si>
-  <si>
     <t>HAKAN DIRAVACI</t>
   </si>
   <si>
-    <t>39821073856</t>
-  </si>
-  <si>
     <t>ŞEYHMUS YEŞİLMEN</t>
   </si>
   <si>
-    <t>14405737652</t>
-  </si>
-  <si>
     <t>ŞADİ TÜRK</t>
   </si>
   <si>
-    <t>16759081108</t>
-  </si>
-  <si>
     <t>NİHAT KIRMIZI</t>
   </si>
   <si>
-    <t>12959987684</t>
-  </si>
-  <si>
     <t>MAHMUT VURAL ERKOÇ</t>
   </si>
   <si>
-    <t>31702544950</t>
-  </si>
-  <si>
     <t>ALİ ACAR</t>
   </si>
   <si>
-    <t>40270324710</t>
-  </si>
-  <si>
     <t>HALE ELPE</t>
   </si>
   <si>
-    <t>13166164660</t>
-  </si>
-  <si>
     <t>ALİM BİLEN</t>
   </si>
   <si>
-    <t>45550717206</t>
-  </si>
-  <si>
     <t>AYŞE GÖKDEMİR</t>
   </si>
   <si>
-    <t>42433490942</t>
-  </si>
-  <si>
     <t>ERCAN ÇÖMEZ</t>
   </si>
   <si>
-    <t>47281826738</t>
-  </si>
-  <si>
     <t>ÇAĞLAYAN YAĞCI</t>
   </si>
   <si>
-    <t>28444998356</t>
-  </si>
-  <si>
     <t>FERİDUN GEÇGEL</t>
   </si>
   <si>
-    <t>44092958696</t>
-  </si>
-  <si>
     <t>MEHMET EMRE ÇAMLIBEL</t>
   </si>
   <si>
-    <t>20468122106</t>
-  </si>
-  <si>
     <t>CANER BİNGÖL</t>
   </si>
   <si>
-    <t>47701654026</t>
-  </si>
-  <si>
     <t>ENES CAN DEMİR</t>
   </si>
   <si>
-    <t>58048559172</t>
-  </si>
-  <si>
     <t>TÜRKER TEKTEN</t>
   </si>
   <si>
-    <t>10487911966</t>
-  </si>
-  <si>
     <t>SALİH TUNCER MUTLUCAN</t>
   </si>
   <si>
-    <t>42379415702</t>
-  </si>
-  <si>
     <t>EGEMEN SÖNMEZ</t>
   </si>
   <si>
-    <t>10546795490</t>
-  </si>
-  <si>
     <t>FATMA BETÜL SAYAN KAYA</t>
   </si>
   <si>
-    <t>61108191816</t>
-  </si>
-  <si>
     <t>İLYAS KAYA</t>
   </si>
   <si>
-    <t>30628668436</t>
+    <t>BAHADIR TONGUÇ</t>
+  </si>
+  <si>
+    <t>MEHMET HAKAN ERDEM</t>
+  </si>
+  <si>
+    <t>MURAT TANRIÖVER</t>
+  </si>
+  <si>
+    <t>ERTAN AYDIN</t>
+  </si>
+  <si>
+    <t>Hüseyin ALTINBAŞ</t>
+  </si>
+  <si>
+    <t>İnan ALTINBAŞ</t>
+  </si>
+  <si>
+    <t>Sami ASLANHAN</t>
+  </si>
+  <si>
+    <t>NABİ KIRMIZI</t>
+  </si>
+  <si>
+    <t>NAZAY TARIM HAYVANCILIK GIDA SANAYİ VE TİCARET LTD ŞTİ</t>
+  </si>
+  <si>
+    <t>SEDAT YILMAZ</t>
+  </si>
+  <si>
+    <t>ÖZCAN GÖNEN</t>
+  </si>
+  <si>
+    <t>ZEYNEL ABİDİN AKÇA</t>
+  </si>
+  <si>
+    <t>HASAN KOÇAK</t>
+  </si>
+  <si>
+    <t>MEHMET GİRAY KOLSUZ</t>
+  </si>
+  <si>
+    <t>ABDULLAH İNAL</t>
+  </si>
+  <si>
+    <t>MUAMMER GEÇGEL</t>
+  </si>
+  <si>
+    <t>İBRAHİM KİLİMCİ</t>
+  </si>
+  <si>
+    <t>AHMET ERDOĞAN</t>
+  </si>
+  <si>
+    <t>AYDIN AŞÇI</t>
+  </si>
+  <si>
+    <t>SUAT YANMAZ</t>
+  </si>
+  <si>
+    <t>ENES TEKE</t>
+  </si>
+  <si>
+    <t>ALİ TURAN YAVUZ</t>
+  </si>
+  <si>
+    <t>MUHAMMED DENİZ</t>
+  </si>
+  <si>
+    <t>NİYAZİ MATPAN</t>
+  </si>
+  <si>
+    <t>SERCAN ERDEM YILMAZ</t>
+  </si>
+  <si>
+    <t>MURAT TARIK ÇELİKKOL</t>
+  </si>
+  <si>
+    <t>MEHMET EROĞLU</t>
+  </si>
+  <si>
+    <t>SAVAŞ ABAK</t>
+  </si>
+  <si>
+    <t>MUSTAFA YUĞAÇ</t>
+  </si>
+  <si>
+    <t>SEVDA KARA</t>
+  </si>
+  <si>
+    <t>ENGİN AYKANAT</t>
+  </si>
+  <si>
+    <t>ABDULSAMET ÇAKIR</t>
+  </si>
+  <si>
+    <t>DİDEM MURADOĞLU</t>
+  </si>
+  <si>
+    <t>AHMET KEREM EREN</t>
+  </si>
+  <si>
+    <t>TALİP ÖZTÜRK</t>
+  </si>
+  <si>
+    <t>TANER DEĞER</t>
+  </si>
+  <si>
+    <t>NECİP ANT FUATOĞLU</t>
+  </si>
+  <si>
+    <t>NACİ TAMER ÖZERDEN</t>
+  </si>
+  <si>
+    <t>ALİ KARABULUT</t>
+  </si>
+  <si>
+    <t>SELÇUK LEKE</t>
+  </si>
+  <si>
+    <t>AHMET TACİR</t>
+  </si>
+  <si>
+    <t>ABDULHAMİT EKTİREN</t>
+  </si>
+  <si>
+    <t>BELİS TACİR</t>
+  </si>
+  <si>
+    <t>CEM EYÜPOĞLU</t>
+  </si>
+  <si>
+    <t>HAŞİM CİHAN YAZGAN</t>
+  </si>
+  <si>
+    <t>BÜLENT AYAZ</t>
+  </si>
+  <si>
+    <t>YÜKSEL KİRİŞÇİOĞLU</t>
+  </si>
+  <si>
+    <t>YILMAZ TÜRKOĞLU</t>
+  </si>
+  <si>
+    <t>CENGİZ DOYRAN</t>
+  </si>
+  <si>
+    <t>ÖMER FARUK ŞAHİN</t>
+  </si>
+  <si>
+    <t>METİN KURU</t>
+  </si>
+  <si>
+    <t>YASİN YURTSEVEN</t>
+  </si>
+  <si>
+    <t>CAHİT ALTAÇLİ</t>
+  </si>
+  <si>
+    <t>AYDIN VELİ SERİN</t>
+  </si>
+  <si>
+    <t>ALİ ÇETE</t>
+  </si>
+  <si>
+    <t>OSMAN BARIŞ ÇEPKEN</t>
+  </si>
+  <si>
+    <t>HASAN HAREZİ</t>
+  </si>
+  <si>
+    <t>MUHAMMED CABİR UĞUR</t>
+  </si>
+  <si>
+    <t>ŞAHİN AYDIN</t>
+  </si>
+  <si>
+    <t>YUSUF TURAN</t>
+  </si>
+  <si>
+    <t>EMİN ELİBÜYÜK</t>
+  </si>
+  <si>
+    <t>MEHMET ALTINBAŞ</t>
+  </si>
+  <si>
+    <t>İBRAHİM TİMUR ÖMÜRGÖNÜLŞEN32584852928</t>
+  </si>
+  <si>
+    <t>ÖNDER GENÇ</t>
+  </si>
+  <si>
+    <t>REZZAN ANIK</t>
+  </si>
+  <si>
+    <t>FATİH TÜRK</t>
+  </si>
+  <si>
+    <t>MURAT BOZDOĞAN</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +808,7 @@
   <dimension ref="A1:G307"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.54296875" customWidth="1"/>
     <col min="3" max="3" width="45.6328125" customWidth="1"/>
     <col min="4" max="4" width="52.1796875" bestFit="1" customWidth="1"/>
@@ -1189,1038 +841,934 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2">
+        <v>17041887022</v>
       </c>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>10</v>
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3">
+        <v>16499328204</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4">
+        <v>27118542178</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>14</v>
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5">
+        <v>18209296322</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>16</v>
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6">
+        <v>38338341250</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>18</v>
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7">
+        <v>38341341186</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>20</v>
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8">
+        <v>46297577726</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>22</v>
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9">
+        <v>14914235908</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>24</v>
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10">
+        <v>13130981972</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>26</v>
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11">
+        <v>6300416499</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>28</v>
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12">
+        <v>40208182498</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>30</v>
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13">
+        <v>59017505046</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>32</v>
+      <c r="A14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14">
+        <v>11531384972</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>34</v>
+      <c r="A15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15">
+        <v>24619559506</v>
       </c>
       <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>36</v>
+      <c r="A16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16">
+        <v>38923077762</v>
       </c>
       <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>38</v>
+      <c r="A17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17">
+        <v>39641173194</v>
       </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>40</v>
+      <c r="A18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18">
+        <v>34460341106</v>
       </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>42</v>
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19">
+        <v>26360128918</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>44</v>
+      <c r="A20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20">
+        <v>65725275188</v>
       </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>46</v>
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21">
+        <v>39136669294</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>48</v>
+      <c r="A22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22">
+        <v>39665042780</v>
       </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>50</v>
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23">
+        <v>29911646312</v>
       </c>
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>52</v>
+      <c r="A24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24">
+        <v>11204630894</v>
       </c>
       <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>54</v>
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25">
+        <v>19811311038</v>
       </c>
       <c r="E25" s="2"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>56</v>
+      <c r="A26" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26">
+        <v>22744032666</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>58</v>
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27">
+        <v>21431395862</v>
       </c>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>60</v>
+      <c r="A28" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28">
+        <v>46843054510</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>62</v>
+      <c r="A29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29">
+        <v>55696312456</v>
       </c>
       <c r="E29" s="2"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>64</v>
+      <c r="A30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30">
+        <v>27880317578</v>
       </c>
       <c r="E30" s="2"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>66</v>
+      <c r="A31" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31">
+        <v>16321768666</v>
       </c>
       <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>68</v>
+      <c r="A32" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32">
+        <v>37582653706</v>
       </c>
       <c r="E32" s="2"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>70</v>
+      <c r="A33" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33">
+        <v>57781224972</v>
       </c>
       <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>72</v>
+      <c r="A34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34">
+        <v>39034066416</v>
       </c>
       <c r="E34" s="2"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>74</v>
+      <c r="A35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35">
+        <v>11245143742</v>
       </c>
       <c r="E35" s="2"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>76</v>
+      <c r="A36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36">
+        <v>33286881896</v>
       </c>
       <c r="E36" s="2"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>78</v>
+      <c r="A37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37">
+        <v>12017322952</v>
       </c>
       <c r="E37" s="3"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>80</v>
+      <c r="A38" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38">
+        <v>10394539734</v>
       </c>
       <c r="E38" s="2"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>82</v>
+      <c r="A39" t="s">
+        <v>90</v>
+      </c>
+      <c r="B39">
+        <v>45295376102</v>
       </c>
       <c r="E39" s="3"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>84</v>
+      <c r="A40" t="s">
+        <v>91</v>
+      </c>
+      <c r="B40">
+        <v>26419103040</v>
       </c>
       <c r="E40" s="2"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>86</v>
+      <c r="A41" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41">
+        <v>11108511862</v>
       </c>
       <c r="E41" s="2"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>88</v>
+      <c r="A42" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42">
+        <v>19451705754</v>
       </c>
       <c r="E42" s="2"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>90</v>
+      <c r="A43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43">
+        <v>31210967234</v>
       </c>
       <c r="E43" s="3"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>92</v>
+      <c r="A44" t="s">
+        <v>95</v>
+      </c>
+      <c r="B44">
+        <v>11477827120</v>
       </c>
       <c r="E44" s="3"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>94</v>
+      <c r="A45" t="s">
+        <v>96</v>
+      </c>
+      <c r="B45">
+        <v>51799172270</v>
       </c>
       <c r="E45" s="3"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>96</v>
+      <c r="A46" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46">
+        <v>15277800796</v>
       </c>
       <c r="E46" s="2"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B47" s="5" t="s">
+      <c r="A47" t="s">
         <v>98</v>
       </c>
+      <c r="B47">
+        <v>49897165188</v>
+      </c>
       <c r="E47" s="2"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
+      <c r="A48" t="s">
         <v>99</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48">
+        <v>20039511056</v>
+      </c>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>100</v>
       </c>
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="4" t="s">
+      <c r="B49">
+        <v>41821346762</v>
+      </c>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>101</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B50">
+        <v>28198182100</v>
+      </c>
+      <c r="E50" s="3"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>102</v>
       </c>
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="4" t="s">
+      <c r="B51">
+        <v>72799076030</v>
+      </c>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>103</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B52">
+        <v>60814502848</v>
+      </c>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>104</v>
       </c>
-      <c r="E50" s="3"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="4" t="s">
+      <c r="B53">
+        <v>30367906554</v>
+      </c>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>105</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B54">
+        <v>24347186678</v>
+      </c>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>106</v>
       </c>
-      <c r="E51" s="2"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="4" t="s">
+      <c r="B55">
+        <v>40681468232</v>
+      </c>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>107</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B56">
+        <v>55084235350</v>
+      </c>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>108</v>
       </c>
-      <c r="E52" s="2"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="4" t="s">
+      <c r="B57">
+        <v>68041121092</v>
+      </c>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>109</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B58">
+        <v>47326336116</v>
+      </c>
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>110</v>
       </c>
-      <c r="E53" s="2"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="4" t="s">
+      <c r="B59">
+        <v>56629694984</v>
+      </c>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>111</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B60">
+        <v>40870522806</v>
+      </c>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>112</v>
       </c>
-      <c r="E54" s="2"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" s="4" t="s">
+      <c r="B61">
+        <v>20596281430</v>
+      </c>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>113</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B62">
+        <v>23518000638</v>
+      </c>
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>114</v>
       </c>
-      <c r="E55" s="2"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" s="4" t="s">
+      <c r="B63">
+        <v>50689313588</v>
+      </c>
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>115</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B64">
+        <v>38305342334</v>
+      </c>
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>116</v>
       </c>
-      <c r="E56" s="2"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" s="4" t="s">
+      <c r="B65" s="5"/>
+      <c r="E65" s="3"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>117</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B66" s="5"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>118</v>
       </c>
-      <c r="E57" s="2"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A58" s="4" t="s">
+      <c r="B67" s="5"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>119</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B68" s="5"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>120</v>
       </c>
-      <c r="E58" s="3"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A59" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E59" s="2"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="E60" s="2"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="E61" s="2"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E62" s="3"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E63" s="3"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="E64" s="3"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A65" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="E65" s="3"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E66" s="2"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A67" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="E67" s="2"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A68" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E68" s="2"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A69" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>142</v>
-      </c>
+      <c r="B69" s="5"/>
       <c r="E69" s="2"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>144</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B70" s="5"/>
       <c r="E70" s="2"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>146</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B71" s="5"/>
       <c r="E71" s="2"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>148</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B72" s="5"/>
       <c r="E72" s="2"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B73" s="5" t="s">
-        <v>150</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B73" s="5"/>
       <c r="E73" s="2"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>152</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B74" s="5"/>
       <c r="E74" s="2"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>154</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B75" s="5"/>
       <c r="E75" s="3"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>156</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B76" s="5"/>
       <c r="E76" s="2"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>158</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B77" s="5"/>
       <c r="E77" s="2"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>160</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B78" s="5"/>
       <c r="E78" s="2"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="B79" s="5" t="s">
-        <v>162</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B79" s="5"/>
       <c r="E79" s="2"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="B80" s="5" t="s">
-        <v>164</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B80" s="5"/>
       <c r="E80" s="2"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>166</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B81" s="5"/>
       <c r="E81" s="3"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>168</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B82" s="5"/>
       <c r="E82" s="2"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>170</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B83" s="5"/>
       <c r="E83" s="2"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>172</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B84" s="5"/>
       <c r="E84" s="2"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>174</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B85" s="5"/>
       <c r="E85" s="2"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>176</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B86" s="5"/>
       <c r="E86" s="2"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>178</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B87" s="5"/>
       <c r="E87" s="2"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>180</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B88" s="5"/>
       <c r="E88" s="2"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>182</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B89" s="5"/>
       <c r="E89" s="2"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>184</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="B90" s="5"/>
       <c r="E90" s="3"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>186</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B91" s="5"/>
       <c r="E91" s="2"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>188</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B92" s="5"/>
       <c r="E92" s="2"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B93" s="5"/>
       <c r="E93" s="3"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>192</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B94" s="5"/>
       <c r="E94" s="3"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>194</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B95" s="5"/>
       <c r="E95" s="3"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B96" s="5" t="s">
-        <v>196</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="B96" s="5"/>
       <c r="E96" s="2"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>198</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B97" s="5"/>
       <c r="E97" s="2"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>200</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B98" s="5"/>
       <c r="E98" s="2"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>202</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B99" s="5"/>
       <c r="E99" s="2"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>204</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B100" s="5"/>
       <c r="E100" s="2"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>206</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B101" s="5"/>
       <c r="E101" s="2"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>208</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B102" s="5"/>
       <c r="E102" s="2"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>210</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B103" s="5"/>
       <c r="E103" s="2"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>212</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="B104" s="5"/>
       <c r="E104" s="2"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>214</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B105" s="5"/>
       <c r="E105" s="2"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>216</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B106" s="5"/>
       <c r="E106" s="2"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>218</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B107" s="5"/>
       <c r="E107" s="3"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="B108" s="5" t="s">
-        <v>220</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B108" s="5"/>
       <c r="E108" s="2"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="B109" s="5" t="s">
-        <v>222</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="B109" s="5"/>
       <c r="E109" s="3"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>224</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="B110" s="5"/>
       <c r="E110" s="2"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>226</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B111" s="5"/>
       <c r="E111" s="2"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>228</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B112" s="5"/>
       <c r="E112" s="2"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>230</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="B113" s="5"/>
       <c r="E113" s="3"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>232</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B114" s="5"/>
       <c r="E114" s="2"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>234</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B115" s="5"/>
       <c r="E115" s="3"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>236</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B116" s="5"/>
       <c r="E116" s="2"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
#261026 fix: fixed global settings
</commit_message>
<xml_diff>
--- a/files/black-list.xlsx
+++ b/files/black-list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koray.zorlu\projects\arierp\arierp_backend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB27AB41-E0D4-4B1D-8C5F-F9883D9393A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF1F6D58-0BE3-4AD8-9185-F2C0FC19DEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BBC1162-E7B6-4495-BD4F-07E3B07D0A73}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>TC/VKN/Pasaport No</t>
   </si>
@@ -59,346 +59,37 @@
     <t>Resmi Gazete Tarih ve Sayısı</t>
   </si>
   <si>
-    <t>GÜL AYŞE ÇOLAK</t>
+    <t>Bayram ÖZATA</t>
   </si>
   <si>
-    <t>MUHAMMED TALHA SAZAK</t>
+    <t>Cihan TUNÇ</t>
   </si>
   <si>
-    <t>OĞUZ TEZMEN</t>
+    <t>Beşir Ömer DEMİR</t>
   </si>
   <si>
-    <t>TOLGA DIRAMALIOL</t>
+    <t>Ümit İlker AVCI</t>
   </si>
   <si>
-    <t>ENVER ÇEVİK</t>
+    <t>Atakay Döviz Sınırlı Yetkili Müessese Anonim Şirketi</t>
   </si>
   <si>
-    <t>MAHMUT KORKMAZ</t>
+    <t>Özgür BÖLÜKBAŞI</t>
   </si>
   <si>
-    <t>MUHAMMED YARIZ</t>
+    <t>SADULLAH ERGÜN</t>
   </si>
   <si>
-    <t>ABDULLAH ERCAN</t>
+    <t>Zekeriya YASEMİN</t>
   </si>
   <si>
-    <t>MELİS SANDAL</t>
+    <t>Cemil Vasken BARIN</t>
   </si>
   <si>
-    <t>EMRULLAH ERCAN</t>
+    <t>UĞUR KURTULAN</t>
   </si>
   <si>
-    <t>ÖMER BEDİR ÇETİNEL</t>
-  </si>
-  <si>
-    <t>MUSTAFA DEDİK</t>
-  </si>
-  <si>
-    <t>HAKAN YILDIZ</t>
-  </si>
-  <si>
-    <t>ENVER GEÇGEL</t>
-  </si>
-  <si>
-    <t>İSMET ÖĞÜT</t>
-  </si>
-  <si>
-    <t>TARZAN TARIK SARVAN</t>
-  </si>
-  <si>
-    <t>TOLGA AYDİN</t>
-  </si>
-  <si>
-    <t>EZGİ KAYA</t>
-  </si>
-  <si>
-    <t>BURHAN TUNÇ ÖZKAN</t>
-  </si>
-  <si>
-    <t>MEHMET SELÇUK AKSOY</t>
-  </si>
-  <si>
-    <t>TURGAY CEYLANİ</t>
-  </si>
-  <si>
-    <t>RIZA KANDEMİR</t>
-  </si>
-  <si>
-    <t>CENGİZ AVCI</t>
-  </si>
-  <si>
-    <t>FURKAN TALAY</t>
-  </si>
-  <si>
-    <t>METEHAN ÜLGENER</t>
-  </si>
-  <si>
-    <t>ALİ YILDIZ</t>
-  </si>
-  <si>
-    <t>KAZİM KOCAPINAR</t>
-  </si>
-  <si>
-    <t>HAKAN DIRAVACI</t>
-  </si>
-  <si>
-    <t>ŞEYHMUS YEŞİLMEN</t>
-  </si>
-  <si>
-    <t>ŞADİ TÜRK</t>
-  </si>
-  <si>
-    <t>NİHAT KIRMIZI</t>
-  </si>
-  <si>
-    <t>MAHMUT VURAL ERKOÇ</t>
-  </si>
-  <si>
-    <t>ALİ ACAR</t>
-  </si>
-  <si>
-    <t>HALE ELPE</t>
-  </si>
-  <si>
-    <t>ALİM BİLEN</t>
-  </si>
-  <si>
-    <t>AYŞE GÖKDEMİR</t>
-  </si>
-  <si>
-    <t>ERCAN ÇÖMEZ</t>
-  </si>
-  <si>
-    <t>ÇAĞLAYAN YAĞCI</t>
-  </si>
-  <si>
-    <t>FERİDUN GEÇGEL</t>
-  </si>
-  <si>
-    <t>MEHMET EMRE ÇAMLIBEL</t>
-  </si>
-  <si>
-    <t>CANER BİNGÖL</t>
-  </si>
-  <si>
-    <t>ENES CAN DEMİR</t>
-  </si>
-  <si>
-    <t>TÜRKER TEKTEN</t>
-  </si>
-  <si>
-    <t>SALİH TUNCER MUTLUCAN</t>
-  </si>
-  <si>
-    <t>EGEMEN SÖNMEZ</t>
-  </si>
-  <si>
-    <t>FATMA BETÜL SAYAN KAYA</t>
-  </si>
-  <si>
-    <t>İLYAS KAYA</t>
-  </si>
-  <si>
-    <t>BAHADIR TONGUÇ</t>
-  </si>
-  <si>
-    <t>MEHMET HAKAN ERDEM</t>
-  </si>
-  <si>
-    <t>MURAT TANRIÖVER</t>
-  </si>
-  <si>
-    <t>ERTAN AYDIN</t>
-  </si>
-  <si>
-    <t>Hüseyin ALTINBAŞ</t>
-  </si>
-  <si>
-    <t>İnan ALTINBAŞ</t>
-  </si>
-  <si>
-    <t>Sami ASLANHAN</t>
-  </si>
-  <si>
-    <t>NABİ KIRMIZI</t>
-  </si>
-  <si>
-    <t>NAZAY TARIM HAYVANCILIK GIDA SANAYİ VE TİCARET LTD ŞTİ</t>
-  </si>
-  <si>
-    <t>SEDAT YILMAZ</t>
-  </si>
-  <si>
-    <t>ÖZCAN GÖNEN</t>
-  </si>
-  <si>
-    <t>ZEYNEL ABİDİN AKÇA</t>
-  </si>
-  <si>
-    <t>HASAN KOÇAK</t>
-  </si>
-  <si>
-    <t>MEHMET GİRAY KOLSUZ</t>
-  </si>
-  <si>
-    <t>ABDULLAH İNAL</t>
-  </si>
-  <si>
-    <t>MUAMMER GEÇGEL</t>
-  </si>
-  <si>
-    <t>İBRAHİM KİLİMCİ</t>
-  </si>
-  <si>
-    <t>AHMET ERDOĞAN</t>
-  </si>
-  <si>
-    <t>AYDIN AŞÇI</t>
-  </si>
-  <si>
-    <t>SUAT YANMAZ</t>
-  </si>
-  <si>
-    <t>ENES TEKE</t>
-  </si>
-  <si>
-    <t>ALİ TURAN YAVUZ</t>
-  </si>
-  <si>
-    <t>MUHAMMED DENİZ</t>
-  </si>
-  <si>
-    <t>NİYAZİ MATPAN</t>
-  </si>
-  <si>
-    <t>SERCAN ERDEM YILMAZ</t>
-  </si>
-  <si>
-    <t>MURAT TARIK ÇELİKKOL</t>
-  </si>
-  <si>
-    <t>MEHMET EROĞLU</t>
-  </si>
-  <si>
-    <t>SAVAŞ ABAK</t>
-  </si>
-  <si>
-    <t>MUSTAFA YUĞAÇ</t>
-  </si>
-  <si>
-    <t>SEVDA KARA</t>
-  </si>
-  <si>
-    <t>ENGİN AYKANAT</t>
-  </si>
-  <si>
-    <t>ABDULSAMET ÇAKIR</t>
-  </si>
-  <si>
-    <t>DİDEM MURADOĞLU</t>
-  </si>
-  <si>
-    <t>AHMET KEREM EREN</t>
-  </si>
-  <si>
-    <t>TALİP ÖZTÜRK</t>
-  </si>
-  <si>
-    <t>TANER DEĞER</t>
-  </si>
-  <si>
-    <t>NECİP ANT FUATOĞLU</t>
-  </si>
-  <si>
-    <t>NACİ TAMER ÖZERDEN</t>
-  </si>
-  <si>
-    <t>ALİ KARABULUT</t>
-  </si>
-  <si>
-    <t>SELÇUK LEKE</t>
-  </si>
-  <si>
-    <t>AHMET TACİR</t>
-  </si>
-  <si>
-    <t>ABDULHAMİT EKTİREN</t>
-  </si>
-  <si>
-    <t>BELİS TACİR</t>
-  </si>
-  <si>
-    <t>CEM EYÜPOĞLU</t>
-  </si>
-  <si>
-    <t>HAŞİM CİHAN YAZGAN</t>
-  </si>
-  <si>
-    <t>BÜLENT AYAZ</t>
-  </si>
-  <si>
-    <t>YÜKSEL KİRİŞÇİOĞLU</t>
-  </si>
-  <si>
-    <t>YILMAZ TÜRKOĞLU</t>
-  </si>
-  <si>
-    <t>CENGİZ DOYRAN</t>
-  </si>
-  <si>
-    <t>ÖMER FARUK ŞAHİN</t>
-  </si>
-  <si>
-    <t>METİN KURU</t>
-  </si>
-  <si>
-    <t>YASİN YURTSEVEN</t>
-  </si>
-  <si>
-    <t>CAHİT ALTAÇLİ</t>
-  </si>
-  <si>
-    <t>AYDIN VELİ SERİN</t>
-  </si>
-  <si>
-    <t>ALİ ÇETE</t>
-  </si>
-  <si>
-    <t>OSMAN BARIŞ ÇEPKEN</t>
-  </si>
-  <si>
-    <t>HASAN HAREZİ</t>
-  </si>
-  <si>
-    <t>MUHAMMED CABİR UĞUR</t>
-  </si>
-  <si>
-    <t>ŞAHİN AYDIN</t>
-  </si>
-  <si>
-    <t>YUSUF TURAN</t>
-  </si>
-  <si>
-    <t>EMİN ELİBÜYÜK</t>
-  </si>
-  <si>
-    <t>MEHMET ALTINBAŞ</t>
-  </si>
-  <si>
-    <t>İBRAHİM TİMUR ÖMÜRGÖNÜLŞEN32584852928</t>
-  </si>
-  <si>
-    <t>ÖNDER GENÇ</t>
-  </si>
-  <si>
-    <t>REZZAN ANIK</t>
-  </si>
-  <si>
-    <t>FATİH TÜRK</t>
-  </si>
-  <si>
-    <t>MURAT BOZDOĞAN</t>
+    <t>İLHAMİ KAYMAK</t>
   </si>
 </sst>
 </file>
@@ -842,932 +533,511 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="B2">
-        <v>17041887022</v>
+        <v>42241503506</v>
       </c>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>16499328204</v>
+        <v>11825140406</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="B4">
-        <v>27118542178</v>
+        <v>19271246024</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="B5">
-        <v>18209296322</v>
+        <v>37123552918</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="B6">
-        <v>38338341250</v>
+        <v>950059257</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="B7">
-        <v>38341341186</v>
+        <v>13195120484</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="B8">
-        <v>46297577726</v>
+        <v>50719176152</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B9">
-        <v>14914235908</v>
+        <v>14774236688</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B10">
-        <v>13130981972</v>
+        <v>20102829330</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B11">
-        <v>6300416499</v>
+        <v>35902504110</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="B12">
-        <v>40208182498</v>
+        <v>20528244748</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13">
-        <v>59017505046</v>
-      </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14">
-        <v>11531384972</v>
-      </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15">
-        <v>24619559506</v>
-      </c>
       <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B16">
-        <v>38923077762</v>
-      </c>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17">
-        <v>39641173194</v>
-      </c>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18">
-        <v>34460341106</v>
-      </c>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19">
-        <v>26360128918</v>
-      </c>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>71</v>
-      </c>
-      <c r="B20">
-        <v>65725275188</v>
-      </c>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>72</v>
-      </c>
-      <c r="B21">
-        <v>39136669294</v>
-      </c>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22">
-        <v>39665042780</v>
-      </c>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>74</v>
-      </c>
-      <c r="B23">
-        <v>29911646312</v>
-      </c>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24">
-        <v>11204630894</v>
-      </c>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25">
-        <v>19811311038</v>
-      </c>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>77</v>
-      </c>
-      <c r="B26">
-        <v>22744032666</v>
-      </c>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27">
-        <v>21431395862</v>
-      </c>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28">
-        <v>46843054510</v>
-      </c>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29">
-        <v>55696312456</v>
-      </c>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30">
-        <v>27880317578</v>
-      </c>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31">
-        <v>16321768666</v>
-      </c>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>83</v>
-      </c>
-      <c r="B32">
-        <v>37582653706</v>
-      </c>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E32" s="2"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33">
-        <v>57781224972</v>
-      </c>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E33" s="2"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34">
-        <v>39034066416</v>
-      </c>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>86</v>
-      </c>
-      <c r="B35">
-        <v>11245143742</v>
-      </c>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36">
-        <v>33286881896</v>
-      </c>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>88</v>
-      </c>
-      <c r="B37">
-        <v>12017322952</v>
-      </c>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>89</v>
-      </c>
-      <c r="B38">
-        <v>10394539734</v>
-      </c>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>90</v>
-      </c>
-      <c r="B39">
-        <v>45295376102</v>
-      </c>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>91</v>
-      </c>
-      <c r="B40">
-        <v>26419103040</v>
-      </c>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>92</v>
-      </c>
-      <c r="B41">
-        <v>11108511862</v>
-      </c>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E41" s="2"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>93</v>
-      </c>
-      <c r="B42">
-        <v>19451705754</v>
-      </c>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E42" s="2"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>94</v>
-      </c>
-      <c r="B43">
-        <v>31210967234</v>
-      </c>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>95</v>
-      </c>
-      <c r="B44">
-        <v>11477827120</v>
-      </c>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>96</v>
-      </c>
-      <c r="B45">
-        <v>51799172270</v>
-      </c>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>97</v>
-      </c>
-      <c r="B46">
-        <v>15277800796</v>
-      </c>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E46" s="2"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>98</v>
-      </c>
-      <c r="B47">
-        <v>49897165188</v>
-      </c>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>99</v>
-      </c>
-      <c r="B48">
-        <v>20039511056</v>
-      </c>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E48" s="2"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>100</v>
-      </c>
-      <c r="B49">
-        <v>41821346762</v>
-      </c>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E49" s="2"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>101</v>
-      </c>
-      <c r="B50">
-        <v>28198182100</v>
-      </c>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>102</v>
-      </c>
-      <c r="B51">
-        <v>72799076030</v>
-      </c>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>103</v>
-      </c>
-      <c r="B52">
-        <v>60814502848</v>
-      </c>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>104</v>
-      </c>
-      <c r="B53">
-        <v>30367906554</v>
-      </c>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>105</v>
-      </c>
-      <c r="B54">
-        <v>24347186678</v>
-      </c>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>106</v>
-      </c>
-      <c r="B55">
-        <v>40681468232</v>
-      </c>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>107</v>
-      </c>
-      <c r="B56">
-        <v>55084235350</v>
-      </c>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>108</v>
-      </c>
-      <c r="B57">
-        <v>68041121092</v>
-      </c>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>109</v>
-      </c>
-      <c r="B58">
-        <v>47326336116</v>
-      </c>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>110</v>
-      </c>
-      <c r="B59">
-        <v>56629694984</v>
-      </c>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E59" s="2"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>111</v>
-      </c>
-      <c r="B60">
-        <v>40870522806</v>
-      </c>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E60" s="2"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>112</v>
-      </c>
-      <c r="B61">
-        <v>20596281430</v>
-      </c>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E61" s="2"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>113</v>
-      </c>
-      <c r="B62">
-        <v>23518000638</v>
-      </c>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>114</v>
-      </c>
-      <c r="B63">
-        <v>50689313588</v>
-      </c>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>115</v>
-      </c>
-      <c r="B64">
-        <v>38305342334</v>
-      </c>
+    <row r="64" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E64" s="3"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>116</v>
-      </c>
       <c r="B65" s="5"/>
       <c r="E65" s="3"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>117</v>
-      </c>
       <c r="B66" s="5"/>
       <c r="E66" s="2"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>118</v>
-      </c>
       <c r="B67" s="5"/>
       <c r="E67" s="2"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>119</v>
-      </c>
       <c r="B68" s="5"/>
       <c r="E68" s="2"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>120</v>
-      </c>
       <c r="B69" s="5"/>
       <c r="E69" s="2"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A70" s="4" t="s">
-        <v>7</v>
-      </c>
+      <c r="A70" s="4"/>
       <c r="B70" s="5"/>
       <c r="E70" s="2"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A71" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="A71" s="4"/>
       <c r="B71" s="5"/>
       <c r="E71" s="2"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A72" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A72" s="4"/>
       <c r="B72" s="5"/>
       <c r="E72" s="2"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73" s="4" t="s">
-        <v>10</v>
-      </c>
+      <c r="A73" s="4"/>
       <c r="B73" s="5"/>
       <c r="E73" s="2"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A74" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="A74" s="4"/>
       <c r="B74" s="5"/>
       <c r="E74" s="2"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A75" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A75" s="4"/>
       <c r="B75" s="5"/>
       <c r="E75" s="3"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A76" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="A76" s="4"/>
       <c r="B76" s="5"/>
       <c r="E76" s="2"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="A77" s="4"/>
       <c r="B77" s="5"/>
       <c r="E77" s="2"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A78" s="4"/>
       <c r="B78" s="5"/>
       <c r="E78" s="2"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A79" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A79" s="4"/>
       <c r="B79" s="5"/>
       <c r="E79" s="2"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A80" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="A80" s="4"/>
       <c r="B80" s="5"/>
       <c r="E80" s="2"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A81" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="A81" s="4"/>
       <c r="B81" s="5"/>
       <c r="E81" s="3"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A82" s="4" t="s">
-        <v>19</v>
-      </c>
+      <c r="A82" s="4"/>
       <c r="B82" s="5"/>
       <c r="E82" s="2"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A83" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="A83" s="4"/>
       <c r="B83" s="5"/>
       <c r="E83" s="2"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84" s="4" t="s">
-        <v>21</v>
-      </c>
+      <c r="A84" s="4"/>
       <c r="B84" s="5"/>
       <c r="E84" s="2"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A85" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="A85" s="4"/>
       <c r="B85" s="5"/>
       <c r="E85" s="2"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A86" s="4" t="s">
-        <v>23</v>
-      </c>
+      <c r="A86" s="4"/>
       <c r="B86" s="5"/>
       <c r="E86" s="2"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A87" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="A87" s="4"/>
       <c r="B87" s="5"/>
       <c r="E87" s="2"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="A88" s="4"/>
       <c r="B88" s="5"/>
       <c r="E88" s="2"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A89" s="4" t="s">
-        <v>26</v>
-      </c>
+      <c r="A89" s="4"/>
       <c r="B89" s="5"/>
       <c r="E89" s="2"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="A90" s="4"/>
       <c r="B90" s="5"/>
       <c r="E90" s="3"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91" s="4" t="s">
-        <v>28</v>
-      </c>
+      <c r="A91" s="4"/>
       <c r="B91" s="5"/>
       <c r="E91" s="2"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92" s="4" t="s">
-        <v>29</v>
-      </c>
+      <c r="A92" s="4"/>
       <c r="B92" s="5"/>
       <c r="E92" s="2"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93" s="4" t="s">
-        <v>30</v>
-      </c>
+      <c r="A93" s="4"/>
       <c r="B93" s="5"/>
       <c r="E93" s="3"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A94" s="4" t="s">
-        <v>31</v>
-      </c>
+      <c r="A94" s="4"/>
       <c r="B94" s="5"/>
       <c r="E94" s="3"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="A95" s="4"/>
       <c r="B95" s="5"/>
       <c r="E95" s="3"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="A96" s="4"/>
       <c r="B96" s="5"/>
       <c r="E96" s="2"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A97" s="4" t="s">
-        <v>34</v>
-      </c>
+      <c r="A97" s="4"/>
       <c r="B97" s="5"/>
       <c r="E97" s="2"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A98" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="A98" s="4"/>
       <c r="B98" s="5"/>
       <c r="E98" s="2"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="A99" s="4"/>
       <c r="B99" s="5"/>
       <c r="E99" s="2"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A100" s="4"/>
       <c r="B100" s="5"/>
       <c r="E100" s="2"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A101" s="4" t="s">
-        <v>38</v>
-      </c>
+      <c r="A101" s="4"/>
       <c r="B101" s="5"/>
       <c r="E101" s="2"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A102" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="A102" s="4"/>
       <c r="B102" s="5"/>
       <c r="E102" s="2"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" s="4" t="s">
-        <v>40</v>
-      </c>
+      <c r="A103" s="4"/>
       <c r="B103" s="5"/>
       <c r="E103" s="2"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="A104" s="4"/>
       <c r="B104" s="5"/>
       <c r="E104" s="2"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" s="4" t="s">
-        <v>42</v>
-      </c>
+      <c r="A105" s="4"/>
       <c r="B105" s="5"/>
       <c r="E105" s="2"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A106" s="4" t="s">
-        <v>43</v>
-      </c>
+      <c r="A106" s="4"/>
       <c r="B106" s="5"/>
       <c r="E106" s="2"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A107" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="A107" s="4"/>
       <c r="B107" s="5"/>
       <c r="E107" s="3"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A108" s="4" t="s">
-        <v>45</v>
-      </c>
+      <c r="A108" s="4"/>
       <c r="B108" s="5"/>
       <c r="E108" s="2"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A109" s="4" t="s">
-        <v>46</v>
-      </c>
+      <c r="A109" s="4"/>
       <c r="B109" s="5"/>
       <c r="E109" s="3"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A110" s="4" t="s">
-        <v>47</v>
-      </c>
+      <c r="A110" s="4"/>
       <c r="B110" s="5"/>
       <c r="E110" s="2"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A111" s="4" t="s">
-        <v>48</v>
-      </c>
+      <c r="A111" s="4"/>
       <c r="B111" s="5"/>
       <c r="E111" s="2"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A112" s="4" t="s">
-        <v>49</v>
-      </c>
+      <c r="A112" s="4"/>
       <c r="B112" s="5"/>
       <c r="E112" s="2"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A113" s="4" t="s">
-        <v>50</v>
-      </c>
+      <c r="A113" s="4"/>
       <c r="B113" s="5"/>
       <c r="E113" s="3"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A114" s="4" t="s">
-        <v>51</v>
-      </c>
+      <c r="A114" s="4"/>
       <c r="B114" s="5"/>
       <c r="E114" s="2"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A115" s="4" t="s">
-        <v>52</v>
-      </c>
+      <c r="A115" s="4"/>
       <c r="B115" s="5"/>
       <c r="E115" s="3"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A116" s="4" t="s">
-        <v>53</v>
-      </c>
+      <c r="A116" s="4"/>
       <c r="B116" s="5"/>
       <c r="E116" s="2"/>
     </row>

</xml_diff>

<commit_message>
#261027 fix: fixed global settings
</commit_message>
<xml_diff>
--- a/files/black-list.xlsx
+++ b/files/black-list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koray.zorlu\projects\arierp\arierp_backend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF1F6D58-0BE3-4AD8-9185-F2C0FC19DEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6D63F7-127F-4FE7-8B6F-6CF9FB5A1EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BBC1162-E7B6-4495-BD4F-07E3B07D0A73}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>TC/VKN/Pasaport No</t>
   </si>
@@ -59,37 +59,43 @@
     <t>Resmi Gazete Tarih ve Sayısı</t>
   </si>
   <si>
-    <t>Bayram ÖZATA</t>
+    <t>Macit İlyas EFENDİOĞLU</t>
   </si>
   <si>
-    <t>Cihan TUNÇ</t>
+    <t>Muhammed Taha KHAN</t>
   </si>
   <si>
-    <t>Beşir Ömer DEMİR</t>
+    <t>Monther ALSALEM</t>
   </si>
   <si>
-    <t>Ümit İlker AVCI</t>
+    <t>Abbas HAIDER</t>
   </si>
   <si>
-    <t>Atakay Döviz Sınırlı Yetkili Müessese Anonim Şirketi</t>
+    <t>Manal MOSSAD ELHAMDI MOHAMED AZAM</t>
   </si>
   <si>
-    <t>Özgür BÖLÜKBAŞI</t>
+    <t>Mohamed NOURELDEEN TAHA ALI MOSTAFA</t>
   </si>
   <si>
-    <t>SADULLAH ERGÜN</t>
+    <t>Safkan Restaurant İşletmeciliği İnşaat Ticaret Limited Şirketi</t>
   </si>
   <si>
-    <t>Zekeriya YASEMİN</t>
+    <t>Ayar Petrol Taşımacılık Ve Turizm Dış Ticaret Limited Şirketi</t>
   </si>
   <si>
-    <t>Cemil Vasken BARIN</t>
+    <t>Barış Akademik Özel Eğitim Hizmetleri Ve Danışmanlık Anonim Şirketi</t>
   </si>
   <si>
-    <t>UĞUR KURTULAN</t>
+    <t>Mct Investment Yapı Anonim Şirketi</t>
   </si>
   <si>
-    <t>İLHAMİ KAYMAK</t>
+    <t xml:space="preserve">Tayo Gayrımenkul Danışmanlığı Limited Şirketi </t>
+  </si>
+  <si>
+    <t>Warsı Investment Yapı Anonim Şirketi</t>
+  </si>
+  <si>
+    <t>Headguarter Uluslararası Yatırım İş Geliştirme Dış Ticaret Limited Şirketi</t>
   </si>
 </sst>
 </file>
@@ -155,13 +161,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,108 +539,114 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2">
-        <v>42241503506</v>
+      <c r="B2" s="6">
+        <v>42065180556</v>
       </c>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3">
-        <v>11825140406</v>
+      <c r="B3" s="6">
+        <v>68863291508</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4">
-        <v>19271246024</v>
+      <c r="B4" s="6">
+        <v>72709161092</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B5">
-        <v>37123552918</v>
+      <c r="B5" s="6">
+        <v>99843652736</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B6">
-        <v>950059257</v>
+      <c r="B6" s="6">
+        <v>99294450912</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B7">
-        <v>13195120484</v>
+      <c r="B7" s="6">
+        <v>99822285320</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8">
-        <v>50719176152</v>
+      <c r="B8" s="6">
+        <v>737052769</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9">
-        <v>14774236688</v>
+      <c r="B9" s="6">
+        <v>1080825319</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B10">
-        <v>20102829330</v>
+      <c r="B10" s="6">
+        <v>1421371774</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B11">
-        <v>35902504110</v>
+      <c r="B11" s="6">
+        <v>7510410627</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B12">
-        <v>20528244748</v>
+      <c r="B12" s="6">
+        <v>8330850311</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
+        <v>19</v>
+      </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>